<commit_message>
resolved merge conflicts, edited withdrawn status
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-27_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-27_Test_Cases.xlsx
@@ -8,26 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samis\OneDrive\Documents\Is212spm\IS212-1\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_B9682CCA0321CFEED1415E3E0547BAF6AB5276F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F28345C-C84D-4348-888D-978248DDDA9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="TC01" sheetId="2" r:id="rId2"/>
-    <sheet name="TC02" sheetId="3" r:id="rId3"/>
-    <sheet name="TC03" sheetId="4" r:id="rId4"/>
-    <sheet name="TC04" sheetId="5" r:id="rId5"/>
-    <sheet name="TC05" sheetId="6" r:id="rId6"/>
-    <sheet name="TC06" sheetId="7" r:id="rId7"/>
-    <sheet name="TC07" sheetId="8" r:id="rId8"/>
+    <sheet name="TC01" sheetId="3" r:id="rId2"/>
+    <sheet name="TC02" sheetId="4" r:id="rId3"/>
+    <sheet name="TC03" sheetId="5" r:id="rId4"/>
+    <sheet name="TC04" sheetId="6" r:id="rId5"/>
+    <sheet name="TC05" sheetId="7" r:id="rId6"/>
+    <sheet name="TC06" sheetId="8" r:id="rId7"/>
+    <sheet name="TC07" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="96">
   <si>
     <t>Story</t>
   </si>
@@ -89,7 +89,7 @@
     <t>SPM-27-TC03</t>
   </si>
   <si>
-    <t>Choosing 'Keep request' in the withdraw dialog leaves the status unchanged</t>
+    <t>Choosing 'Keep request' in the withdrawal dialog leaves the status unchanged</t>
   </si>
   <si>
     <t>AC2</t>
@@ -107,7 +107,7 @@
     <t>SPM-27-TC04</t>
   </si>
   <si>
-    <t>Organiser withdraws a Submitted or Under review request</t>
+    <t>Coordinator records a withdrawal and the organiser sees Withdrawn</t>
   </si>
   <si>
     <t>AC2, AC3</t>
@@ -119,7 +119,7 @@
     <t>SPM-27-TC05</t>
   </si>
   <si>
-    <t>Organiser has no way to change the status of an event from Approved onwards</t>
+    <t>Organiser has no way to change the status of their event</t>
   </si>
   <si>
     <t>AC4</t>
@@ -134,10 +134,7 @@
     <t>SPM-27-TC06</t>
   </si>
   <si>
-    <t>Only the event's organiser is offered 'Withdraw request'</t>
-  </si>
-  <si>
-    <t>AC3</t>
+    <t>Only the assigned coordinator is offered 'Record withdrawal'</t>
   </si>
   <si>
     <t>TC07</t>
@@ -174,15 +171,18 @@
     <t>SPM-27-TC02
 SPM-27-TC03
 SPM-27-TC04
+SPM-27-TC06
 SPM-27-TC07</t>
   </si>
   <si>
+    <t>AC3</t>
+  </si>
+  <si>
     <t>The system displays appropriate statuses such as Submitted, Under Review, Approved, Planning, Confirmed, Completed, Rejected, Postponed, Withdrawn or Cancelled.</t>
   </si>
   <si>
     <t>SPM-27-TC01
-SPM-27-TC04
-SPM-27-TC06</t>
+SPM-27-TC04</t>
   </si>
   <si>
     <t>The Event Organiser cannot manually change the event status.</t>
@@ -203,8 +203,9 @@
 src/app/venues/search/page.tsx
 docs/ConnectSphere_Status_Lifecycle.drawio
 docs/PERMISSIONS.md
-scripts/seed-spm30.ts
-prisma/seed.ts</t>
+scripts/seed-spm27.ts
+prisma/seed.ts
+src/app/queue/page.tsx</t>
   </si>
   <si>
     <t>Item</t>
@@ -220,8 +221,7 @@
     <t>Test Steps</t>
   </si>
   <si>
-    <t>1. Click 'My Events' in the sidebar
-2. Find each of the 14 SPM27 events in the list and read its Status column</t>
+    <t>1. Click 'My Events' in the sidebar</t>
   </si>
   <si>
     <t>Test Data</t>
@@ -233,9 +233,7 @@
     <t>Expected Result</t>
   </si>
   <si>
-    <t>Each of the 14 SPM27 events shows a coloured status badge with exactly the label listed in Test data, so all 10 statuses appear: Submitted, Under review, Approved, Planning, Confirmed, Completed, Rejected, Postponed, Withdrawn, Cancelled (some on more than one event).
-No status is shown as a raw value such as 'under_review'.
-Only Bayu Energy Partners events are listed; no other company's events appear.</t>
+    <t>Step 1: Each of the 14 SPM27 events shows a coloured status badge with exactly the label listed in Test data, so all 10 statuses appear: Submitted, Under review, Approved, Planning, Confirmed, Completed, Rejected, Postponed, Withdrawn, Cancelled (some on more than one event). No status is shown as a raw value such as 'under_review'. Only Bayu Energy Partners events are listed; no other company's events appear.</t>
   </si>
   <si>
     <t>Created By</t>
@@ -253,133 +251,155 @@
     <t>Pass/Fail/Not Executed/Blocked</t>
   </si>
   <si>
-    <t>Pass</t>
-  </si>
-  <si>
     <t>Remarks</t>
   </si>
   <si>
-    <t>NA</t>
-  </si>
-  <si>
     <t>Executed by</t>
   </si>
   <si>
-    <t>Sammi</t>
-  </si>
-  <si>
     <t>Date of Execution</t>
   </si>
   <si>
-    <t>Test data freshly loaded: run `npm run fixtures:spm27` from the project folder just before this case.
+    <t>Test data freshly loaded: run `npm run fixtures:spm27` from the project folder before and after this case.
 'SPM27 Bayu Investor Day' is Submitted with no coordinator.
 Accounts: Hakim Zulkifli (hakim.zulkifli@bayuenergypa.com / password123), Event Organiser; Grace Lim (grace.lim@connectsphere.com / password123), Event Operations Manager.</t>
   </si>
   <si>
-    <t>1. Log in as Hakim Zulkifli and open 'SPM27 Bayu Investor Day' from 'My Events'
-2. Read the badge under the title and the 'Status' row in the 'Details' card
-3. Log out and log in as Grace Lim
-4. Click 'Assignments' in the sidebar
-5. On the 'SPM27 Bayu Investor Day' row, choose 'Hui Shan Neo' in 'Assign to' and click 'Assign'
+    <t>1. Log in as Hakim Zulkifli
+2. Click 'My Events' in the sidebar
+3. Open 'SPM27 Bayu Investor Day'
+4. Log out and log in as Grace Lim
+5. Click 'Assignments' in the sidebar
+6. On the 'SPM27 Bayu Investor Day' row, choose 'Hui Shan Neo' in 'Assign to'
+7. Click 'Assign'
+8. Log out and log in as Hakim Zulkifli
+9. Click 'My Events' in the sidebar
+10. Open 'SPM27 Bayu Investor Day'</t>
+  </si>
+  <si>
+    <t>Event: SPM27 Bayu Investor Day | Coordinator: Hui Shan Neo</t>
+  </si>
+  <si>
+    <t>Step 3: The badge under the title and the Details 'Status' row both read 'Submitted'.
+Step 10: The badge and the Details 'Status' row both read 'Under review'.</t>
+  </si>
+  <si>
+    <t>Test data freshly loaded: run `npm run fixtures:spm27` from the project folder just before this case.
+'SPM27 Bayu Grid Workshop' is Under review, coordinator Hui Shan Neo.
+Logged in as Hui Shan Neo (huishan.neo@connectsphere.com / password123), Event Coordinator.
+Withdrawal follows customer clarification #103: the organiser asks the Event Coordinator outside the system, and the assigned coordinator records the withdrawal while the request is Under review. Withdrawn is final.</t>
+  </si>
+  <si>
+    <t>1. Click 'All Events' in the sidebar
+2. Open 'SPM27 Bayu Grid Workshop'
+3. Click 'Record withdrawal'
+4. In the dialog, click 'Keep request'
+5. Reload the page</t>
+  </si>
+  <si>
+    <t>Event: SPM27 Bayu Grid Workshop (Under review)</t>
+  </si>
+  <si>
+    <t>Step 3: A dialog titled 'Record this withdrawal?' appears.
+Step 4: The dialog closes.
+Step 5: The badge still reads 'Under review' and the 'Record withdrawal' button is still shown.</t>
+  </si>
+  <si>
+    <t>Test data freshly loaded: run `npm run fixtures:spm27` from the project folder before and after this case (SPM-27-TC03 does not change the data, so this case can run straight after it).
+'SPM27 Bayu Grid Workshop' is Under review, coordinator Hui Shan Neo.
+Accounts: Hui Shan Neo (huishan.neo@connectsphere.com / password123), Event Coordinator; Hakim Zulkifli (hakim.zulkifli@bayuenergypa.com / password123), Event Organiser.
+Withdrawal follows customer clarification #103: the organiser asks the Event Coordinator outside the system, and the assigned coordinator records the withdrawal while the request is Under review. Withdrawn is final.</t>
+  </si>
+  <si>
+    <t>1. Log in as Hui Shan Neo
+2. Click 'All Events' in the sidebar
+3. Open 'SPM27 Bayu Grid Workshop'
+4. Click 'Record withdrawal'
+5. In the dialog 'Record this withdrawal?', click 'Record withdrawal'
 6. Log out and log in as Hakim Zulkifli
-7. Click 'My Events' and open 'SPM27 Bayu Investor Day'</t>
-  </si>
-  <si>
-    <t>Event: SPM27 Bayu Investor Day | Coordinator: Hui Shan Neo</t>
-  </si>
-  <si>
-    <t>Before the assignment, the header badge and the Details 'Status' row both read 'Submitted'.
-After the assignment, both read 'Under review'.</t>
-  </si>
-  <si>
-    <t>Test data freshly loaded: run `npm run fixtures:spm27` from the project folder just before this case.
-'SPM27 Bayu Safety Briefing' is Submitted.
-Logged in as Hakim Zulkifli (hakim.zulkifli@bayuenergypa.com / password123).</t>
-  </si>
-  <si>
-    <t>1. Click 'My Events' and open 'SPM27 Bayu Safety Briefing'
-2. Click 'Withdraw request'
-3. In the dialog 'Withdraw this request?', click 'Keep request'
-4. Reload the page</t>
-  </si>
-  <si>
-    <t>Event: SPM27 Bayu Safety Briefing (Submitted)</t>
-  </si>
-  <si>
-    <t>The dialog closes.
-After reloading, the badge still reads 'Submitted' and the 'Withdraw request' button is still shown.</t>
-  </si>
-  <si>
-    <t>Test data freshly loaded: run `npm run fixtures:spm27` from the project folder (TC03 does not change the data, so it can run straight after TC03).
-'SPM27 Bayu Safety Briefing' is Submitted; 'SPM27 Bayu Grid Workshop' is Under review (coordinator Hui Shan Neo).
-Logged in as Hakim Zulkifli (hakim.zulkifli@bayuenergypa.com / password123).
-Team decision: see TC03.</t>
-  </si>
-  <si>
-    <t>1. Click 'My Events' and open 'SPM27 Bayu Safety Briefing'
-2. Click 'Withdraw request'
-3. In the dialog 'Withdraw this request?', click 'Withdraw request'
-4. Repeat steps 1-3 for 'SPM27 Bayu Grid Workshop'</t>
-  </si>
-  <si>
-    <t>Submitted: SPM27 Bayu Safety Briefing | Under review: SPM27 Bayu Grid Workshop</t>
-  </si>
-  <si>
-    <t>For each event, the success message 'Your request has been withdrawn.' is shown and the status badge changes to 'Withdrawn'.</t>
+7. Click 'My Events' in the sidebar
+8. Open 'SPM27 Bayu Grid Workshop'</t>
+  </si>
+  <si>
+    <t>Step 5: The message 'The withdrawal has been recorded.' is shown, the badge changes to 'Withdrawn' and the 'Record withdrawal' button is gone.
+Step 8: The badge and the Details 'Status' row read 'Withdrawn'.</t>
   </si>
   <si>
     <t>Test data loaded: run `npm run fixtures:spm27` from the project folder if it has not been run for this test pass.
 Logged in as Hakim Zulkifli (hakim.zulkifli@bayuenergypa.com / password123).</t>
   </si>
   <si>
-    <t>1. Click 'My Events' and open 'SPM27 Bayu Supplier Day'
-2. Look for 'Withdraw request' or any button, dropdown or field that changes the status
-3. Repeat for every other event in Test data</t>
-  </si>
-  <si>
-    <t>Approved (first status after the withdraw window closes): SPM27 Bayu Supplier Day | Planning: SPM27 Bayu Leadership Retreat | Confirmed: SPM27 Bayu Annual Conference | Postponed: SPM27 Bayu Community Fair | Completed: SPM27 Bayu Graduate Induction | Rejected: SPM27 Bayu Overnight Site Visit | Cancelled: SPM27 Bayu Product Showcase | Withdrawn: SPM27 Bayu Partner Lunch</t>
-  </si>
-  <si>
-    <t>On every event the status is shown only as the badge and the read-only Details 'Status' row.
-No 'Withdraw request' button is shown, and there is no button, dropdown or field that changes the status.</t>
-  </si>
-  <si>
     <t>Test data freshly loaded: run `npm run fixtures:spm27` from the project folder just before this case.
-'SPM27 Bayu Town Hall' is Submitted with no coordinator; 'SPM27 Bayu Contractor Briefing' is Under review with coordinator Hui Shan Neo.
-Team decision: see TC03.</t>
+'SPM27 Bayu Contractor Briefing' is Under review with coordinator Hui Shan Neo; 'SPM27 Bayu Supplier Day' is Approved with coordinator Hui Shan Neo.
+Withdrawal follows customer clarification #103: the organiser asks the Event Coordinator outside the system, and the assigned coordinator records the withdrawal while the request is Under review. Withdrawn is final.</t>
   </si>
   <si>
     <t>1. Log in as Grace Lim (grace.lim@connectsphere.com / password123)
-2. Click 'All Events' and open 'SPM27 Bayu Town Hall'
-3. Look for a 'Withdraw request' button
-4. Log out and log in as Hui Shan Neo (huishan.neo@connectsphere.com / password123)
-5. Click 'All Events' and open 'SPM27 Bayu Contractor Briefing'
-6. Look for a 'Withdraw request' button</t>
-  </si>
-  <si>
-    <t>Event Operations Manager: grace.lim@connectsphere.com / password123 | Event Coordinator: huishan.neo@connectsphere.com / password123</t>
-  </si>
-  <si>
-    <t>Neither user sees a 'Withdraw request' button.</t>
+2. Click 'All Events' in the sidebar
+3. Open 'SPM27 Bayu Contractor Briefing'
+4. Log out and log in as Daniel Tan (daniel.tan@connectsphere.com / password123)
+5. Click 'All Events' in the sidebar
+6. Open 'SPM27 Bayu Contractor Briefing'
+7. Log out and log in as Hui Shan Neo (huishan.neo@connectsphere.com / password123)
+8. Click 'All Events' in the sidebar
+9. Open 'SPM27 Bayu Supplier Day'</t>
+  </si>
+  <si>
+    <t>Event Operations Manager: Grace Lim | Unassigned Event Coordinator: Daniel Tan | Assigned Event Coordinator: Hui Shan Neo | Under review: SPM27 Bayu Contractor Briefing | Approved: SPM27 Bayu Supplier Day</t>
+  </si>
+  <si>
+    <t>Step 3: No 'Record withdrawal' button is shown.
+Step 6: No 'Record withdrawal' button is shown.
+Step 9: No 'Record withdrawal' button is shown, because the event is past review.</t>
   </si>
   <si>
     <t>Test data loaded: run `npm run fixtures:spm27` from the project folder if it has not been run for this test pass.
-'SPM27 Bayu Partner Lunch' was withdrawn while Submitted (no coordinator); 'SPM27 Bayu Wind Farm Tour' was withdrawn while Under review (coordinator Hui Shan Neo).</t>
-  </si>
-  <si>
-    <t>1. Log in as Grace Lim (grace.lim@connectsphere.com / password123)
-2. Click 'Assignments' in the sidebar and look for 'SPM27 Bayu Partner Lunch' in 'Awaiting assignment'
-3. Click 'All Events' and open 'SPM27 Bayu Partner Lunch'
-4. Log out and log in as Hui Shan Neo (huishan.neo@connectsphere.com / password123)
-5. Click 'All Events' and open 'SPM27 Bayu Wind Farm Tour'
-6. Open the 'Equipment' tab</t>
-  </si>
-  <si>
-    <t>Withdrawn from Submitted: SPM27 Bayu Partner Lunch | Withdrawn from Under review: SPM27 Bayu Wind Farm Tour</t>
-  </si>
-  <si>
-    <t>'SPM27 Bayu Partner Lunch' is not in the 'Awaiting assignment' list, and its event page has no 'Assign a coordinator' card.
-The Equipment tab of 'SPM27 Bayu Wind Farm Tour' shows 'This event is withdrawn — equipment requirements can no longer be changed.' with no add, edit or remove controls.</t>
+'SPM27 Bayu Partner Lunch' and 'SPM27 Bayu Wind Farm Tour' were withdrawn while Under review (coordinator Hui Shan Neo).</t>
+  </si>
+  <si>
+    <t>1. Log in as Hui Shan Neo (huishan.neo@connectsphere.com / password123)
+2. Click 'Review Queue' in the sidebar
+3. Click 'All Events' in the sidebar
+4. Open 'SPM27 Bayu Wind Farm Tour'
+5. Open the 'Equipment' tab</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Sammi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click 'My Events' in the sidebar
+2. Open 'SPM27 Bayu Safety Briefing'
+3. Click 'My Events' in the sidebar
+4. Open 'SPM27 Bayu Contractor Briefing'
+5. Click 'My Events' in the sidebar
+6. Open 'SPM27 Bayu Supplier Day'
+7. Click 'My Events' in the sidebar
+8. Open 'SPM27 Bayu Leadership Retreat'
+</t>
+  </si>
+  <si>
+    <t>Submitted: SPM27 Bayu Safety Briefing | Under review: SPM27 Bayu Contractor Briefing | Approved: SPM27 Bayu Supplier Day | Planning: SPM27 Bayu Leadership Retreat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Step 2: On 'SPM27 Bayu Safety Briefing', the status is shown only as the badge and the read-only Details 'Status' row; there is no 'Record withdrawal' button and no button, dropdown or field that changes the status.
+Step 4: On 'SPM27 Bayu Contractor Briefing', the status is shown only as the badge and the read-only Details 'Status' row; there is no 'Record withdrawal' button and no button, dropdown or field that changes the status.
+Step 6: On 'SPM27 Bayu Supplier Day', the status is shown only as the badge and the read-only Details 'Status' row; there is no 'Record withdrawal' button and no button, dropdown or field that changes the status.
+Step 8: On 'SPM27 Bayu Leadership Retreat', the status is shown only as the badge and the read-only Details 'Status' row; there is no 'Record withdrawal' button and no button, dropdown or field that changes the status.
+</t>
+  </si>
+  <si>
+    <t>Withdrawn: SPM27 Bayu Wind Farm Tour</t>
+  </si>
+  <si>
+    <t>Step 2:  'SPM27 Bayu Wind Farm Tour' is not listed.
+Step 4: The badge reads 'Withdrawn' and there is no 'Record withdrawal' or 'Review request' action.
+Step 5: The tab shows 'This event is withdrawn — equipment requirements can no longer be changed.' with no add, edit or remove controls.</t>
   </si>
 </sst>
 </file>
@@ -547,12 +567,12 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -770,7 +790,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -785,7 +805,7 @@
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="16" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="14"/>
@@ -793,7 +813,7 @@
       <c r="E1" s="14"/>
       <c r="F1" s="15"/>
     </row>
-    <row r="3" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="13" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
@@ -813,7 +833,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="25" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
@@ -833,7 +853,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="25" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>14</v>
       </c>
@@ -853,7 +873,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="25" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>18</v>
       </c>
@@ -893,7 +913,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>28</v>
       </c>
@@ -913,7 +933,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="25" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>33</v>
       </c>
@@ -924,7 +944,7 @@
         <v>35</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>22</v>
@@ -933,15 +953,15 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="25" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="C10" s="9" t="s">
         <v>38</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>39</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>21</v>
@@ -953,110 +973,102 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-    </row>
-    <row r="14" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+    <row r="13" spans="1:6" ht="13" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="16" t="s">
         <v>40</v>
       </c>
+      <c r="C13" s="14"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="15"/>
+    </row>
+    <row r="14" spans="1:6" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>42</v>
+      </c>
       <c r="B14" s="13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="15"/>
       <c r="E14" s="13" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F14" s="15"/>
     </row>
-    <row r="15" spans="1:6" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B15" s="16" t="s">
-        <v>44</v>
+        <v>21</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>45</v>
       </c>
       <c r="C15" s="14"/>
       <c r="D15" s="15"/>
-      <c r="E15" s="16" t="s">
-        <v>45</v>
+      <c r="E15" s="13" t="s">
+        <v>46</v>
       </c>
       <c r="F15" s="15"/>
     </row>
-    <row r="16" spans="1:6" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" s="16" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>48</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="15"/>
-      <c r="E16" s="16" t="s">
-        <v>47</v>
+      <c r="E16" s="13" t="s">
+        <v>49</v>
       </c>
       <c r="F16" s="15"/>
     </row>
-    <row r="17" spans="1:6" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>48</v>
+        <v>31</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>50</v>
       </c>
       <c r="C17" s="14"/>
       <c r="D17" s="15"/>
-      <c r="E17" s="16" t="s">
-        <v>49</v>
+      <c r="E17" s="13" t="s">
+        <v>29</v>
       </c>
       <c r="F17" s="15"/>
     </row>
-    <row r="18" spans="1:6" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="F18" s="15"/>
-    </row>
-    <row r="20" spans="1:6" ht="193" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
+    <row r="19" spans="1:6" ht="206.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B19" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="15"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="E14:F14"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="B15:D15"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="B16:D16"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="E15:F15"/>
-    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B19:F19"/>
     <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="B16:D16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'TC01'!A1" display="TC01" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -1072,132 +1084,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" s="2"/>
-    </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="B8" s="12">
-        <v>46297</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="6"/>
-    </row>
-    <row r="11" spans="1:3" ht="100" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B15" s="12">
-        <v>46297</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -1209,7 +1095,7 @@
     <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>53</v>
       </c>
@@ -1220,39 +1106,39 @@
         <v>3</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>54</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>58</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>60</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1263,7 +1149,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>64</v>
       </c>
@@ -1271,48 +1157,48 @@
         <v>46297</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>53</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="6"/>
     </row>
-    <row r="11" spans="1:3" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="87.5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>66</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="B13" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B14" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>69</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="B15" s="12">
         <v>46297</v>
@@ -1323,7 +1209,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -1335,7 +1221,7 @@
     <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>53</v>
       </c>
@@ -1346,23 +1232,23 @@
         <v>3</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="62.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>54</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1370,15 +1256,15 @@
         <v>58</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>60</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1389,7 +1275,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>64</v>
       </c>
@@ -1397,48 +1283,48 @@
         <v>46297</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>53</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="6"/>
     </row>
-    <row r="11" spans="1:3" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="50" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>66</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="B13" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B14" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>69</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="B15" s="12">
         <v>46297</v>
@@ -1449,7 +1335,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -1461,7 +1347,7 @@
     <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>53</v>
       </c>
@@ -1472,15 +1358,15 @@
         <v>3</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>54</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1488,23 +1374,23 @@
         <v>56</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>58</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>60</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1515,7 +1401,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>64</v>
       </c>
@@ -1523,48 +1409,48 @@
         <v>46297</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>53</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="6"/>
     </row>
-    <row r="11" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="50" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>66</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="B13" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B14" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>69</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="B15" s="12">
         <v>46297</v>
@@ -1575,7 +1461,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -1587,7 +1473,7 @@
     <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>53</v>
       </c>
@@ -1598,39 +1484,39 @@
         <v>3</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="179.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>54</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>58</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>60</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1641,7 +1527,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>64</v>
       </c>
@@ -1649,48 +1535,48 @@
         <v>46297</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>53</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="6"/>
     </row>
-    <row r="11" spans="1:3" ht="50" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="50" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>66</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="B13" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B14" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>69</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="B15" s="12">
         <v>46297</v>
@@ -1701,7 +1587,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -1713,7 +1599,7 @@
     <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>53</v>
       </c>
@@ -1724,39 +1610,39 @@
         <v>3</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>54</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>58</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="212.5" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>60</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1767,7 +1653,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>64</v>
       </c>
@@ -1775,48 +1661,48 @@
         <v>46297</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>53</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="6"/>
     </row>
-    <row r="11" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="212.5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>66</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="B13" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B14" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>69</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="B15" s="12">
         <v>46297</v>
@@ -1827,7 +1713,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -1839,7 +1725,7 @@
     <col min="2" max="2" width="56.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>53</v>
       </c>
@@ -1850,23 +1736,149 @@
         <v>3</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>54</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>56</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>94</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" s="12">
+        <v>46297</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="6"/>
+    </row>
+    <row r="11" spans="1:3" ht="50" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B15" s="12">
+        <v>46297</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.81640625" customWidth="1"/>
+    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="2"/>
+    </row>
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
@@ -1874,15 +1886,15 @@
         <v>58</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>60</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1893,7 +1905,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>64</v>
       </c>
@@ -1901,48 +1913,48 @@
         <v>46297</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="13" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>53</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="6"/>
     </row>
-    <row r="11" spans="1:3" ht="62.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>66</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="B13" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B14" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>69</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="12.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="B15" s="12">
         <v>46297</v>

</xml_diff>